<commit_message>
Aggiunti i segnali decodificati nel 'ID'
</commit_message>
<xml_diff>
--- a/Resources/ALU Operations.xlsx
+++ b/Resources/ALU Operations.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Il mio Drive\Architetture Digitali Avanzate\CPU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Il mio Drive\Architetture Digitali Avanzate\CPU\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B263F1E-6424-4B23-BAF2-3D1F7C2A3610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F56B783-A2D4-4EAB-89D9-6D5D26C35B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{06DEFF1A-5186-46E6-B88F-5F33049B43C5}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="11640" xr2:uid="{06DEFF1A-5186-46E6-B88F-5F33049B43C5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Arithmetic-Logic" sheetId="1" r:id="rId1"/>
-    <sheet name="Branch" sheetId="2" r:id="rId2"/>
+    <sheet name="Convenzioni di formato" sheetId="3" r:id="rId1"/>
+    <sheet name="Arithmetic-Logic" sheetId="1" r:id="rId2"/>
+    <sheet name="Branch" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="71">
   <si>
     <t>14       12</t>
   </si>
@@ -184,6 +185,72 @@
   </si>
   <si>
     <t>11                7</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>func7</t>
+  </si>
+  <si>
+    <t>Imm[11:0]</t>
+  </si>
+  <si>
+    <t>rs2</t>
+  </si>
+  <si>
+    <t>rs1</t>
+  </si>
+  <si>
+    <t>func3</t>
+  </si>
+  <si>
+    <t>rd</t>
+  </si>
+  <si>
+    <t>opcode</t>
+  </si>
+  <si>
+    <t>Imm[31:12]</t>
+  </si>
+  <si>
+    <t>Imm[20|10:1|11|19:12]</t>
+  </si>
+  <si>
+    <t>POS BITs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#BITs </t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Imm[11:5]</t>
+  </si>
+  <si>
+    <t>imm[4:0]</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>31 [ 30                             20]  19[18                  12]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1   [                 12                  ]   1 [              7          ] </t>
   </si>
 </sst>
 </file>
@@ -191,9 +258,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="165" formatCode="0000"/>
-    <numFmt numFmtId="166" formatCode="0000000"/>
-    <numFmt numFmtId="167" formatCode="000"/>
+    <numFmt numFmtId="164" formatCode="0000"/>
+    <numFmt numFmtId="165" formatCode="0000000"/>
+    <numFmt numFmtId="166" formatCode="000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -232,7 +299,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -582,11 +649,126 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -636,6 +818,123 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -645,12 +944,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -666,96 +959,57 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1069,6 +1323,272 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE765E64-1BA4-4E0C-B65E-51C6045EDF8A}">
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="83"/>
+    <col min="2" max="2" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="58" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="60"/>
+    </row>
+    <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="61" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="62"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
+    </row>
+    <row r="4" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="61">
+        <v>20</v>
+      </c>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="60"/>
+    </row>
+    <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="48" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="40" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B7" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="52" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B8" s="54" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="55"/>
+      <c r="D8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="53" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B9" s="51" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="50" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="53" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B10" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="53" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B11" s="56" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="57"/>
+      <c r="D11" s="57"/>
+      <c r="E11" s="57"/>
+      <c r="F11" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G11" s="53" t="s">
+        <v>56</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="66" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="67"/>
+      <c r="D12" s="67"/>
+      <c r="E12" s="67"/>
+      <c r="F12" s="68" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" s="69" t="s">
+        <v>56</v>
+      </c>
+      <c r="H12" s="70" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="84" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="79" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="81"/>
+      <c r="F13" s="71"/>
+      <c r="G13" s="73"/>
+      <c r="H13" s="74"/>
+    </row>
+    <row r="14" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="85" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" s="80" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="76"/>
+      <c r="D14" s="76"/>
+      <c r="E14" s="82"/>
+      <c r="F14" s="75"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="78"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="86"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B12:E12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C1842B-3C4E-484C-9319-072FB30D1681}">
   <dimension ref="B1:K26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1083,45 +1603,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="19"/>
-      <c r="J1" s="17" t="s">
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="60"/>
+      <c r="J1" s="58" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="19"/>
+      <c r="K1" s="60"/>
     </row>
     <row r="2" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="61" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="19"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="60"/>
       <c r="J2" s="10" t="s">
         <v>36</v>
       </c>
       <c r="K2" s="12"/>
     </row>
     <row r="3" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="22">
+      <c r="B3" s="61">
         <v>20</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="19"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
       <c r="J3" s="10" t="s">
         <v>37</v>
       </c>
@@ -1130,7 +1650,7 @@
       </c>
     </row>
     <row r="4" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -1139,17 +1659,17 @@
       <c r="D4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="E4" s="25" t="s">
         <v>29</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="39" t="s">
+      <c r="G4" s="30" t="s">
         <v>27</v>
       </c>
       <c r="H4" s="12"/>
-      <c r="J4" s="27">
+      <c r="J4" s="18">
         <v>0</v>
       </c>
       <c r="K4" s="8" t="s">
@@ -1157,7 +1677,7 @@
       </c>
     </row>
     <row r="5" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="21" t="s">
         <v>33</v>
       </c>
       <c r="C5" s="11" t="s">
@@ -1166,19 +1686,19 @@
       <c r="D5" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="34" t="s">
+      <c r="E5" s="25" t="s">
         <v>0</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="40" t="s">
+      <c r="G5" s="31" t="s">
         <v>34</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="27">
+      <c r="J5" s="18">
         <v>1000</v>
       </c>
       <c r="K5" s="8" t="s">
@@ -1186,26 +1706,26 @@
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="26"/>
+      <c r="C6" s="65"/>
       <c r="D6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="35">
+      <c r="E6" s="26">
         <v>0</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="41">
+      <c r="G6" s="32">
         <v>10011</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="J6" s="27">
+      <c r="J6" s="18">
         <v>1</v>
       </c>
       <c r="K6" s="7" t="s">
@@ -1213,7 +1733,7 @@
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B7" s="31">
+      <c r="B7" s="22">
         <v>0</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -1222,19 +1742,19 @@
       <c r="D7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="36">
+      <c r="E7" s="27">
         <v>1</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G7" s="42">
+      <c r="G7" s="33">
         <v>10011</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="J7" s="27">
+      <c r="J7" s="18">
         <v>10</v>
       </c>
       <c r="K7" s="8" t="s">
@@ -1242,26 +1762,26 @@
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="21"/>
+      <c r="C8" s="57"/>
       <c r="D8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="36">
+      <c r="E8" s="27">
         <v>10</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="42">
+      <c r="G8" s="33">
         <v>10011</v>
       </c>
       <c r="H8" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="J8" s="27">
+      <c r="J8" s="18">
         <v>11</v>
       </c>
       <c r="K8" s="8" t="s">
@@ -1269,26 +1789,26 @@
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="21"/>
+      <c r="C9" s="57"/>
       <c r="D9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="36">
+      <c r="E9" s="27">
         <v>11</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G9" s="42">
+      <c r="G9" s="33">
         <v>10011</v>
       </c>
       <c r="H9" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="J9" s="27">
+      <c r="J9" s="18">
         <v>100</v>
       </c>
       <c r="K9" s="8" t="s">
@@ -1296,26 +1816,26 @@
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="21"/>
+      <c r="C10" s="57"/>
       <c r="D10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="28">
         <v>100</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G10" s="42">
+      <c r="G10" s="33">
         <v>10011</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="J10" s="27">
+      <c r="J10" s="18">
         <v>101</v>
       </c>
       <c r="K10" s="8" t="s">
@@ -1323,7 +1843,7 @@
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B11" s="31">
+      <c r="B11" s="22">
         <v>0</v>
       </c>
       <c r="C11" s="4" t="s">
@@ -1332,19 +1852,19 @@
       <c r="D11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="36">
+      <c r="E11" s="27">
         <v>101</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="42">
+      <c r="G11" s="33">
         <v>10011</v>
       </c>
       <c r="H11" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="J11" s="27">
+      <c r="J11" s="18">
         <v>1101</v>
       </c>
       <c r="K11" s="8" t="s">
@@ -1352,7 +1872,7 @@
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="31">
+      <c r="B12" s="22">
         <v>100000</v>
       </c>
       <c r="C12" s="4" t="s">
@@ -1361,19 +1881,19 @@
       <c r="D12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="36">
+      <c r="E12" s="27">
         <v>101</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="42">
+      <c r="G12" s="33">
         <v>10011</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="J12" s="27">
+      <c r="J12" s="18">
         <v>110</v>
       </c>
       <c r="K12" s="8" t="s">
@@ -1381,26 +1901,26 @@
       </c>
     </row>
     <row r="13" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="21"/>
+      <c r="C13" s="57"/>
       <c r="D13" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="36">
+      <c r="E13" s="27">
         <v>110</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G13" s="42">
+      <c r="G13" s="33">
         <v>10011</v>
       </c>
       <c r="H13" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="J13" s="28">
+      <c r="J13" s="19">
         <v>111</v>
       </c>
       <c r="K13" s="9" t="s">
@@ -1408,20 +1928,20 @@
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="21"/>
+      <c r="C14" s="57"/>
       <c r="D14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="36">
+      <c r="E14" s="27">
         <v>111</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G14" s="42">
+      <c r="G14" s="33">
         <v>10011</v>
       </c>
       <c r="H14" s="15" t="s">
@@ -1429,7 +1949,7 @@
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B15" s="31">
+      <c r="B15" s="22">
         <v>0</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -1438,13 +1958,13 @@
       <c r="D15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="36">
+      <c r="E15" s="27">
         <v>0</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="42">
+      <c r="G15" s="33">
         <v>110011</v>
       </c>
       <c r="H15" s="15" t="s">
@@ -1452,7 +1972,7 @@
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B16" s="31">
+      <c r="B16" s="22">
         <v>100000</v>
       </c>
       <c r="C16" s="4" t="s">
@@ -1461,13 +1981,13 @@
       <c r="D16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="36">
+      <c r="E16" s="27">
         <v>0</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="42">
+      <c r="G16" s="33">
         <v>110011</v>
       </c>
       <c r="H16" s="15" t="s">
@@ -1475,7 +1995,7 @@
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B17" s="31">
+      <c r="B17" s="22">
         <v>0</v>
       </c>
       <c r="C17" s="4" t="s">
@@ -1484,13 +2004,13 @@
       <c r="D17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="36">
+      <c r="E17" s="27">
         <v>1</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G17" s="42">
+      <c r="G17" s="33">
         <v>110011</v>
       </c>
       <c r="H17" s="14" t="s">
@@ -1498,7 +2018,7 @@
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B18" s="31">
+      <c r="B18" s="22">
         <v>0</v>
       </c>
       <c r="C18" s="4" t="s">
@@ -1507,13 +2027,13 @@
       <c r="D18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="36">
+      <c r="E18" s="27">
         <v>10</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G18" s="42">
+      <c r="G18" s="33">
         <v>110011</v>
       </c>
       <c r="H18" s="15" t="s">
@@ -1521,7 +2041,7 @@
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B19" s="31">
+      <c r="B19" s="22">
         <v>0</v>
       </c>
       <c r="C19" s="4" t="s">
@@ -1530,13 +2050,13 @@
       <c r="D19" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="36">
+      <c r="E19" s="27">
         <v>11</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G19" s="42">
+      <c r="G19" s="33">
         <v>110011</v>
       </c>
       <c r="H19" s="15" t="s">
@@ -1544,7 +2064,7 @@
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B20" s="31">
+      <c r="B20" s="22">
         <v>0</v>
       </c>
       <c r="C20" s="4" t="s">
@@ -1553,13 +2073,13 @@
       <c r="D20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="37">
+      <c r="E20" s="28">
         <v>100</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G20" s="42">
+      <c r="G20" s="33">
         <v>110011</v>
       </c>
       <c r="H20" s="15" t="s">
@@ -1567,7 +2087,7 @@
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B21" s="31">
+      <c r="B21" s="22">
         <v>0</v>
       </c>
       <c r="C21" s="4" t="s">
@@ -1576,13 +2096,13 @@
       <c r="D21" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="36">
+      <c r="E21" s="27">
         <v>101</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G21" s="42">
+      <c r="G21" s="33">
         <v>110011</v>
       </c>
       <c r="H21" s="15" t="s">
@@ -1590,7 +2110,7 @@
       </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B22" s="31">
+      <c r="B22" s="22">
         <v>100000</v>
       </c>
       <c r="C22" s="4" t="s">
@@ -1599,13 +2119,13 @@
       <c r="D22" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E22" s="36">
+      <c r="E22" s="27">
         <v>101</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G22" s="42">
+      <c r="G22" s="33">
         <v>110011</v>
       </c>
       <c r="H22" s="15" t="s">
@@ -1613,7 +2133,7 @@
       </c>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B23" s="31">
+      <c r="B23" s="22">
         <v>0</v>
       </c>
       <c r="C23" s="4" t="s">
@@ -1622,13 +2142,13 @@
       <c r="D23" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E23" s="36">
+      <c r="E23" s="27">
         <v>110</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G23" s="42">
+      <c r="G23" s="33">
         <v>110011</v>
       </c>
       <c r="H23" s="15" t="s">
@@ -1636,7 +2156,7 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="32">
+      <c r="B24" s="23">
         <v>0</v>
       </c>
       <c r="C24" s="6" t="s">
@@ -1645,13 +2165,13 @@
       <c r="D24" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E24" s="38">
+      <c r="E24" s="29">
         <v>111</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G24" s="43">
+      <c r="G24" s="34">
         <v>110011</v>
       </c>
       <c r="H24" s="16" t="s">
@@ -1671,12 +2191,12 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="D2:H2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1685,55 +2205,55 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6B22D93-4160-4CE6-8BAE-21BC001536C2}">
   <dimension ref="B1:I12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.21875" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" style="20" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.21875" style="33" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" style="24" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5546875" style="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="19"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="60"/>
     </row>
     <row r="3" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="61" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="19"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="60"/>
     </row>
     <row r="4" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="22">
+      <c r="B4" s="61">
         <v>20</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="19"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="60"/>
     </row>
     <row r="5" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="11" t="s">
@@ -1742,42 +2262,42 @@
       <c r="D5" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="34" t="s">
+      <c r="E5" s="25" t="s">
         <v>29</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="39" t="s">
+      <c r="G5" s="30" t="s">
         <v>27</v>
       </c>
       <c r="H5" s="12"/>
     </row>
     <row r="6" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="47" t="s">
+      <c r="C6" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="47" t="s">
+      <c r="D6" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="48" t="s">
+      <c r="E6" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="47" t="s">
+      <c r="F6" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="57" t="s">
+      <c r="G6" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="49" t="s">
+      <c r="H6" s="40" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="35" t="s">
         <v>40</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -1786,21 +2306,21 @@
       <c r="D7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="35">
+      <c r="E7" s="26">
         <v>0</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="51">
+      <c r="G7" s="42">
         <v>1100011</v>
       </c>
-      <c r="H7" s="52" t="s">
+      <c r="H7" s="43" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="22" t="s">
         <v>40</v>
       </c>
       <c r="C8" s="4" t="s">
@@ -1809,21 +2329,21 @@
       <c r="D8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="36">
+      <c r="E8" s="27">
         <v>1</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="50">
+      <c r="G8" s="41">
         <v>1100011</v>
       </c>
-      <c r="H8" s="53" t="s">
+      <c r="H8" s="44" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="22" t="s">
         <v>40</v>
       </c>
       <c r="C9" s="4" t="s">
@@ -1832,21 +2352,21 @@
       <c r="D9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="36">
+      <c r="E9" s="27">
         <v>100</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="50">
+      <c r="G9" s="41">
         <v>1100011</v>
       </c>
-      <c r="H9" s="54" t="s">
+      <c r="H9" s="45" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="22" t="s">
         <v>40</v>
       </c>
       <c r="C10" s="4" t="s">
@@ -1855,22 +2375,22 @@
       <c r="D10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="36">
+      <c r="E10" s="27">
         <v>101</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="50">
+      <c r="G10" s="41">
         <v>1100011</v>
       </c>
-      <c r="H10" s="53" t="s">
+      <c r="H10" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="I10" s="58"/>
+      <c r="I10" s="49"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="22" t="s">
         <v>40</v>
       </c>
       <c r="C11" s="4" t="s">
@@ -1879,21 +2399,21 @@
       <c r="D11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="36">
+      <c r="E11" s="27">
         <v>110</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="50">
+      <c r="G11" s="41">
         <v>1100011</v>
       </c>
-      <c r="H11" s="53" t="s">
+      <c r="H11" s="44" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="12" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="23" t="s">
         <v>40</v>
       </c>
       <c r="C12" s="6" t="s">
@@ -1902,16 +2422,16 @@
       <c r="D12" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="45">
+      <c r="E12" s="36">
         <v>111</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="55">
+      <c r="G12" s="46">
         <v>1100011</v>
       </c>
-      <c r="H12" s="56" t="s">
+      <c r="H12" s="47" t="s">
         <v>47</v>
       </c>
     </row>

</xml_diff>